<commit_message>
fix: correct file paths in payment generators and regenerate all sample Excel files
</commit_message>
<xml_diff>
--- a/backend/excel-files/results_computer_science_sem1.xlsx
+++ b/backend/excel-files/results_computer_science_sem1.xlsx
@@ -425,10 +425,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>UMaT/PG/0015/22</v>
+        <v>UMaT/PG/0003/22</v>
       </c>
       <c r="B2" t="str">
-        <v>Ekua Acheampong</v>
+        <v>Mensah Agyei</v>
       </c>
       <c r="C2" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -437,15 +437,15 @@
         <v>3</v>
       </c>
       <c r="E2">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>UMaT/PG/0015/22</v>
+        <v>UMaT/PG/0003/22</v>
       </c>
       <c r="B3" t="str">
-        <v>Ekua Acheampong</v>
+        <v>Mensah Agyei</v>
       </c>
       <c r="C3" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -454,15 +454,15 @@
         <v>3</v>
       </c>
       <c r="E3">
-        <v>40</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>UMaT/PG/0015/22</v>
+        <v>UMaT/PG/0003/22</v>
       </c>
       <c r="B4" t="str">
-        <v>Ekua Acheampong</v>
+        <v>Mensah Agyei</v>
       </c>
       <c r="C4" t="str">
         <v>Realtime Systems</v>
@@ -471,15 +471,15 @@
         <v>3</v>
       </c>
       <c r="E4">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>UMaT/PG/0015/22</v>
+        <v>UMaT/PG/0003/22</v>
       </c>
       <c r="B5" t="str">
-        <v>Ekua Acheampong</v>
+        <v>Mensah Agyei</v>
       </c>
       <c r="C5" t="str">
         <v>Parallel Computing</v>
@@ -488,15 +488,15 @@
         <v>3</v>
       </c>
       <c r="E5">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>UMaT/PG/0018/22</v>
+        <v>UMaT/PG/0008/22</v>
       </c>
       <c r="B6" t="str">
-        <v>Akua Sarpong</v>
+        <v>Kwabena Ofori</v>
       </c>
       <c r="C6" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -505,15 +505,15 @@
         <v>3</v>
       </c>
       <c r="E6">
-        <v>79</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>UMaT/PG/0018/22</v>
+        <v>UMaT/PG/0008/22</v>
       </c>
       <c r="B7" t="str">
-        <v>Akua Sarpong</v>
+        <v>Kwabena Ofori</v>
       </c>
       <c r="C7" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -522,15 +522,15 @@
         <v>3</v>
       </c>
       <c r="E7">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>UMaT/PG/0018/22</v>
+        <v>UMaT/PG/0008/22</v>
       </c>
       <c r="B8" t="str">
-        <v>Akua Sarpong</v>
+        <v>Kwabena Ofori</v>
       </c>
       <c r="C8" t="str">
         <v>Realtime Systems</v>
@@ -539,15 +539,15 @@
         <v>3</v>
       </c>
       <c r="E8">
-        <v>93</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>UMaT/PG/0018/22</v>
+        <v>UMaT/PG/0008/22</v>
       </c>
       <c r="B9" t="str">
-        <v>Akua Sarpong</v>
+        <v>Kwabena Ofori</v>
       </c>
       <c r="C9" t="str">
         <v>Parallel Computing</v>
@@ -556,15 +556,15 @@
         <v>3</v>
       </c>
       <c r="E9">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>UMaT/PG/0023/22</v>
+        <v>UMaT/PG/0009/22</v>
       </c>
       <c r="B10" t="str">
-        <v>Kodwo Ofori</v>
+        <v>Panyin Darko</v>
       </c>
       <c r="C10" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -573,15 +573,15 @@
         <v>3</v>
       </c>
       <c r="E10">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>UMaT/PG/0023/22</v>
+        <v>UMaT/PG/0009/22</v>
       </c>
       <c r="B11" t="str">
-        <v>Kodwo Ofori</v>
+        <v>Panyin Darko</v>
       </c>
       <c r="C11" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -590,15 +590,15 @@
         <v>3</v>
       </c>
       <c r="E11">
-        <v>94</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>UMaT/PG/0023/22</v>
+        <v>UMaT/PG/0009/22</v>
       </c>
       <c r="B12" t="str">
-        <v>Kodwo Ofori</v>
+        <v>Panyin Darko</v>
       </c>
       <c r="C12" t="str">
         <v>Realtime Systems</v>
@@ -607,15 +607,15 @@
         <v>3</v>
       </c>
       <c r="E12">
-        <v>78</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>UMaT/PG/0023/22</v>
+        <v>UMaT/PG/0009/22</v>
       </c>
       <c r="B13" t="str">
-        <v>Kodwo Ofori</v>
+        <v>Panyin Darko</v>
       </c>
       <c r="C13" t="str">
         <v>Parallel Computing</v>
@@ -624,15 +624,15 @@
         <v>3</v>
       </c>
       <c r="E13">
-        <v>79</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>UMaT/PG/0029/22</v>
+        <v>UMaT/PG/0015/22</v>
       </c>
       <c r="B14" t="str">
-        <v>Abena Ansah</v>
+        <v>Ebo Mensah</v>
       </c>
       <c r="C14" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -641,15 +641,15 @@
         <v>3</v>
       </c>
       <c r="E14">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>UMaT/PG/0029/22</v>
+        <v>UMaT/PG/0015/22</v>
       </c>
       <c r="B15" t="str">
-        <v>Abena Ansah</v>
+        <v>Ebo Mensah</v>
       </c>
       <c r="C15" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -658,15 +658,15 @@
         <v>3</v>
       </c>
       <c r="E15">
-        <v>66</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>UMaT/PG/0029/22</v>
+        <v>UMaT/PG/0015/22</v>
       </c>
       <c r="B16" t="str">
-        <v>Abena Ansah</v>
+        <v>Ebo Mensah</v>
       </c>
       <c r="C16" t="str">
         <v>Realtime Systems</v>
@@ -675,15 +675,15 @@
         <v>3</v>
       </c>
       <c r="E16">
-        <v>47</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>UMaT/PG/0029/22</v>
+        <v>UMaT/PG/0015/22</v>
       </c>
       <c r="B17" t="str">
-        <v>Abena Ansah</v>
+        <v>Ebo Mensah</v>
       </c>
       <c r="C17" t="str">
         <v>Parallel Computing</v>
@@ -692,15 +692,15 @@
         <v>3</v>
       </c>
       <c r="E17">
-        <v>66</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>UMaT/PG/0054/22</v>
+        <v>UMaT/PG/0042/22</v>
       </c>
       <c r="B18" t="str">
-        <v>Kojo Annan</v>
+        <v>Serwa Darko</v>
       </c>
       <c r="C18" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -709,15 +709,15 @@
         <v>3</v>
       </c>
       <c r="E18">
-        <v>66</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>UMaT/PG/0054/22</v>
+        <v>UMaT/PG/0042/22</v>
       </c>
       <c r="B19" t="str">
-        <v>Kojo Annan</v>
+        <v>Serwa Darko</v>
       </c>
       <c r="C19" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -726,15 +726,15 @@
         <v>3</v>
       </c>
       <c r="E19">
-        <v>70</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>UMaT/PG/0054/22</v>
+        <v>UMaT/PG/0042/22</v>
       </c>
       <c r="B20" t="str">
-        <v>Kojo Annan</v>
+        <v>Serwa Darko</v>
       </c>
       <c r="C20" t="str">
         <v>Realtime Systems</v>
@@ -743,15 +743,15 @@
         <v>3</v>
       </c>
       <c r="E20">
-        <v>47</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>UMaT/PG/0054/22</v>
+        <v>UMaT/PG/0042/22</v>
       </c>
       <c r="B21" t="str">
-        <v>Kojo Annan</v>
+        <v>Serwa Darko</v>
       </c>
       <c r="C21" t="str">
         <v>Parallel Computing</v>
@@ -760,15 +760,15 @@
         <v>3</v>
       </c>
       <c r="E21">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>UMaT/PG/0067/22</v>
+        <v>UMaT/PG/0047/22</v>
       </c>
       <c r="B22" t="str">
-        <v>Kwadwo Darko</v>
+        <v>Mensah Asante</v>
       </c>
       <c r="C22" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -777,15 +777,15 @@
         <v>3</v>
       </c>
       <c r="E22">
-        <v>53</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>UMaT/PG/0067/22</v>
+        <v>UMaT/PG/0047/22</v>
       </c>
       <c r="B23" t="str">
-        <v>Kwadwo Darko</v>
+        <v>Mensah Asante</v>
       </c>
       <c r="C23" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -794,15 +794,15 @@
         <v>3</v>
       </c>
       <c r="E23">
-        <v>86</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>UMaT/PG/0067/22</v>
+        <v>UMaT/PG/0047/22</v>
       </c>
       <c r="B24" t="str">
-        <v>Kwadwo Darko</v>
+        <v>Mensah Asante</v>
       </c>
       <c r="C24" t="str">
         <v>Realtime Systems</v>
@@ -811,15 +811,15 @@
         <v>3</v>
       </c>
       <c r="E24">
-        <v>60</v>
+        <v>83</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>UMaT/PG/0067/22</v>
+        <v>UMaT/PG/0047/22</v>
       </c>
       <c r="B25" t="str">
-        <v>Kwadwo Darko</v>
+        <v>Mensah Asante</v>
       </c>
       <c r="C25" t="str">
         <v>Parallel Computing</v>
@@ -828,15 +828,15 @@
         <v>3</v>
       </c>
       <c r="E25">
-        <v>51</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>UMaT/PG/0073/22</v>
+        <v>UMaT/PG/0064/22</v>
       </c>
       <c r="B26" t="str">
-        <v>Afi Akuffo</v>
+        <v>Akua Danquah</v>
       </c>
       <c r="C26" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -845,15 +845,15 @@
         <v>3</v>
       </c>
       <c r="E26">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>UMaT/PG/0073/22</v>
+        <v>UMaT/PG/0064/22</v>
       </c>
       <c r="B27" t="str">
-        <v>Afi Akuffo</v>
+        <v>Akua Danquah</v>
       </c>
       <c r="C27" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -862,15 +862,15 @@
         <v>3</v>
       </c>
       <c r="E27">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>UMaT/PG/0073/22</v>
+        <v>UMaT/PG/0064/22</v>
       </c>
       <c r="B28" t="str">
-        <v>Afi Akuffo</v>
+        <v>Akua Danquah</v>
       </c>
       <c r="C28" t="str">
         <v>Realtime Systems</v>
@@ -879,15 +879,15 @@
         <v>3</v>
       </c>
       <c r="E28">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>UMaT/PG/0073/22</v>
+        <v>UMaT/PG/0064/22</v>
       </c>
       <c r="B29" t="str">
-        <v>Afi Akuffo</v>
+        <v>Akua Danquah</v>
       </c>
       <c r="C29" t="str">
         <v>Parallel Computing</v>
@@ -896,15 +896,15 @@
         <v>3</v>
       </c>
       <c r="E29">
-        <v>50</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>UMaT/PG/0091/24</v>
+        <v>UMaT/PG/0084/24</v>
       </c>
       <c r="B30" t="str">
-        <v>Esi Adjei</v>
+        <v>Kojo Mensah</v>
       </c>
       <c r="C30" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -913,15 +913,15 @@
         <v>3</v>
       </c>
       <c r="E30">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>UMaT/PG/0091/24</v>
+        <v>UMaT/PG/0084/24</v>
       </c>
       <c r="B31" t="str">
-        <v>Esi Adjei</v>
+        <v>Kojo Mensah</v>
       </c>
       <c r="C31" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -930,15 +930,15 @@
         <v>3</v>
       </c>
       <c r="E31">
-        <v>89</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>UMaT/PG/0091/24</v>
+        <v>UMaT/PG/0084/24</v>
       </c>
       <c r="B32" t="str">
-        <v>Esi Adjei</v>
+        <v>Kojo Mensah</v>
       </c>
       <c r="C32" t="str">
         <v>Realtime Systems</v>
@@ -947,15 +947,15 @@
         <v>3</v>
       </c>
       <c r="E32">
-        <v>75</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>UMaT/PG/0091/24</v>
+        <v>UMaT/PG/0084/24</v>
       </c>
       <c r="B33" t="str">
-        <v>Esi Adjei</v>
+        <v>Kojo Mensah</v>
       </c>
       <c r="C33" t="str">
         <v>Parallel Computing</v>
@@ -964,15 +964,15 @@
         <v>3</v>
       </c>
       <c r="E33">
-        <v>62</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>UMaT/PG/0102/24</v>
+        <v>UMaT/PG/0087/24</v>
       </c>
       <c r="B34" t="str">
-        <v>Yaw Darko</v>
+        <v>Araba Acheampong</v>
       </c>
       <c r="C34" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -981,15 +981,15 @@
         <v>3</v>
       </c>
       <c r="E34">
-        <v>46</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>UMaT/PG/0102/24</v>
+        <v>UMaT/PG/0087/24</v>
       </c>
       <c r="B35" t="str">
-        <v>Yaw Darko</v>
+        <v>Araba Acheampong</v>
       </c>
       <c r="C35" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -998,15 +998,15 @@
         <v>3</v>
       </c>
       <c r="E35">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>UMaT/PG/0102/24</v>
+        <v>UMaT/PG/0087/24</v>
       </c>
       <c r="B36" t="str">
-        <v>Yaw Darko</v>
+        <v>Araba Acheampong</v>
       </c>
       <c r="C36" t="str">
         <v>Realtime Systems</v>
@@ -1015,15 +1015,15 @@
         <v>3</v>
       </c>
       <c r="E36">
-        <v>75</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>UMaT/PG/0102/24</v>
+        <v>UMaT/PG/0087/24</v>
       </c>
       <c r="B37" t="str">
-        <v>Yaw Darko</v>
+        <v>Araba Acheampong</v>
       </c>
       <c r="C37" t="str">
         <v>Parallel Computing</v>
@@ -1032,15 +1032,15 @@
         <v>3</v>
       </c>
       <c r="E37">
-        <v>81</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>UMaT/PG/0116/24</v>
+        <v>UMaT/PG/0096/24</v>
       </c>
       <c r="B38" t="str">
-        <v>Araba Ofori</v>
+        <v>Abena Darko</v>
       </c>
       <c r="C38" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1049,15 +1049,15 @@
         <v>3</v>
       </c>
       <c r="E38">
-        <v>67</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>UMaT/PG/0116/24</v>
+        <v>UMaT/PG/0096/24</v>
       </c>
       <c r="B39" t="str">
-        <v>Araba Ofori</v>
+        <v>Abena Darko</v>
       </c>
       <c r="C39" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1066,15 +1066,15 @@
         <v>3</v>
       </c>
       <c r="E39">
-        <v>90</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>UMaT/PG/0116/24</v>
+        <v>UMaT/PG/0096/24</v>
       </c>
       <c r="B40" t="str">
-        <v>Araba Ofori</v>
+        <v>Abena Darko</v>
       </c>
       <c r="C40" t="str">
         <v>Realtime Systems</v>
@@ -1083,15 +1083,15 @@
         <v>3</v>
       </c>
       <c r="E40">
-        <v>92</v>
+        <v>46</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>UMaT/PG/0116/24</v>
+        <v>UMaT/PG/0096/24</v>
       </c>
       <c r="B41" t="str">
-        <v>Araba Ofori</v>
+        <v>Abena Darko</v>
       </c>
       <c r="C41" t="str">
         <v>Parallel Computing</v>
@@ -1100,15 +1100,15 @@
         <v>3</v>
       </c>
       <c r="E41">
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>UMaT/PG/0148/24</v>
+        <v>UMaT/PG/0097/24</v>
       </c>
       <c r="B42" t="str">
-        <v>Kwaku Annan</v>
+        <v>Serwa Ofori</v>
       </c>
       <c r="C42" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1117,15 +1117,15 @@
         <v>3</v>
       </c>
       <c r="E42">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>UMaT/PG/0148/24</v>
+        <v>UMaT/PG/0097/24</v>
       </c>
       <c r="B43" t="str">
-        <v>Kwaku Annan</v>
+        <v>Serwa Ofori</v>
       </c>
       <c r="C43" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1134,15 +1134,15 @@
         <v>3</v>
       </c>
       <c r="E43">
-        <v>67</v>
+        <v>79</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>UMaT/PG/0148/24</v>
+        <v>UMaT/PG/0097/24</v>
       </c>
       <c r="B44" t="str">
-        <v>Kwaku Annan</v>
+        <v>Serwa Ofori</v>
       </c>
       <c r="C44" t="str">
         <v>Realtime Systems</v>
@@ -1151,15 +1151,15 @@
         <v>3</v>
       </c>
       <c r="E44">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>UMaT/PG/0148/24</v>
+        <v>UMaT/PG/0097/24</v>
       </c>
       <c r="B45" t="str">
-        <v>Kwaku Annan</v>
+        <v>Serwa Ofori</v>
       </c>
       <c r="C45" t="str">
         <v>Parallel Computing</v>
@@ -1168,15 +1168,15 @@
         <v>3</v>
       </c>
       <c r="E45">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>UMaT/PG/0157/24</v>
+        <v>UMaT/PG/0106/24</v>
       </c>
       <c r="B46" t="str">
-        <v>Ama Owusu</v>
+        <v>Serwa Agyei</v>
       </c>
       <c r="C46" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1185,15 +1185,15 @@
         <v>3</v>
       </c>
       <c r="E46">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>UMaT/PG/0157/24</v>
+        <v>UMaT/PG/0106/24</v>
       </c>
       <c r="B47" t="str">
-        <v>Ama Owusu</v>
+        <v>Serwa Agyei</v>
       </c>
       <c r="C47" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1202,15 +1202,15 @@
         <v>3</v>
       </c>
       <c r="E47">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>UMaT/PG/0157/24</v>
+        <v>UMaT/PG/0106/24</v>
       </c>
       <c r="B48" t="str">
-        <v>Ama Owusu</v>
+        <v>Serwa Agyei</v>
       </c>
       <c r="C48" t="str">
         <v>Realtime Systems</v>
@@ -1219,15 +1219,15 @@
         <v>3</v>
       </c>
       <c r="E48">
-        <v>42</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>UMaT/PG/0157/24</v>
+        <v>UMaT/PG/0106/24</v>
       </c>
       <c r="B49" t="str">
-        <v>Ama Owusu</v>
+        <v>Serwa Agyei</v>
       </c>
       <c r="C49" t="str">
         <v>Parallel Computing</v>
@@ -1236,15 +1236,15 @@
         <v>3</v>
       </c>
       <c r="E49">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>UMaT/PG/0159/24</v>
+        <v>UMaT/PG/0113/24</v>
       </c>
       <c r="B50" t="str">
-        <v>Mensah Addo</v>
+        <v>Kwabena Addo</v>
       </c>
       <c r="C50" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1253,15 +1253,15 @@
         <v>3</v>
       </c>
       <c r="E50">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>UMaT/PG/0159/24</v>
+        <v>UMaT/PG/0113/24</v>
       </c>
       <c r="B51" t="str">
-        <v>Mensah Addo</v>
+        <v>Kwabena Addo</v>
       </c>
       <c r="C51" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1270,15 +1270,15 @@
         <v>3</v>
       </c>
       <c r="E51">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>UMaT/PG/0159/24</v>
+        <v>UMaT/PG/0113/24</v>
       </c>
       <c r="B52" t="str">
-        <v>Mensah Addo</v>
+        <v>Kwabena Addo</v>
       </c>
       <c r="C52" t="str">
         <v>Realtime Systems</v>
@@ -1287,15 +1287,15 @@
         <v>3</v>
       </c>
       <c r="E52">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>UMaT/PG/0159/24</v>
+        <v>UMaT/PG/0113/24</v>
       </c>
       <c r="B53" t="str">
-        <v>Mensah Addo</v>
+        <v>Kwabena Addo</v>
       </c>
       <c r="C53" t="str">
         <v>Parallel Computing</v>
@@ -1309,10 +1309,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>UMaT/PG/0186/24</v>
+        <v>UMaT/PG/0121/24</v>
       </c>
       <c r="B54" t="str">
-        <v>Ato Afriyie</v>
+        <v>Yaw Ansah</v>
       </c>
       <c r="C54" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1321,15 +1321,15 @@
         <v>3</v>
       </c>
       <c r="E54">
-        <v>54</v>
+        <v>61</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>UMaT/PG/0186/24</v>
+        <v>UMaT/PG/0121/24</v>
       </c>
       <c r="B55" t="str">
-        <v>Ato Afriyie</v>
+        <v>Yaw Ansah</v>
       </c>
       <c r="C55" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1338,15 +1338,15 @@
         <v>3</v>
       </c>
       <c r="E55">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>UMaT/PG/0186/24</v>
+        <v>UMaT/PG/0121/24</v>
       </c>
       <c r="B56" t="str">
-        <v>Ato Afriyie</v>
+        <v>Yaw Ansah</v>
       </c>
       <c r="C56" t="str">
         <v>Realtime Systems</v>
@@ -1355,15 +1355,15 @@
         <v>3</v>
       </c>
       <c r="E56">
-        <v>62</v>
+        <v>52</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>UMaT/PG/0186/24</v>
+        <v>UMaT/PG/0121/24</v>
       </c>
       <c r="B57" t="str">
-        <v>Ato Afriyie</v>
+        <v>Yaw Ansah</v>
       </c>
       <c r="C57" t="str">
         <v>Parallel Computing</v>
@@ -1372,15 +1372,15 @@
         <v>3</v>
       </c>
       <c r="E57">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>UMaT/PG/0188/24</v>
+        <v>UMaT/PG/0139/24</v>
       </c>
       <c r="B58" t="str">
-        <v>Efua Akuffo</v>
+        <v>Akua Quaye</v>
       </c>
       <c r="C58" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1389,15 +1389,15 @@
         <v>3</v>
       </c>
       <c r="E58">
-        <v>78</v>
+        <v>84</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>UMaT/PG/0188/24</v>
+        <v>UMaT/PG/0139/24</v>
       </c>
       <c r="B59" t="str">
-        <v>Efua Akuffo</v>
+        <v>Akua Quaye</v>
       </c>
       <c r="C59" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1406,15 +1406,15 @@
         <v>3</v>
       </c>
       <c r="E59">
-        <v>50</v>
+        <v>79</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>UMaT/PG/0188/24</v>
+        <v>UMaT/PG/0139/24</v>
       </c>
       <c r="B60" t="str">
-        <v>Efua Akuffo</v>
+        <v>Akua Quaye</v>
       </c>
       <c r="C60" t="str">
         <v>Realtime Systems</v>
@@ -1423,15 +1423,15 @@
         <v>3</v>
       </c>
       <c r="E60">
-        <v>68</v>
+        <v>52</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>UMaT/PG/0188/24</v>
+        <v>UMaT/PG/0139/24</v>
       </c>
       <c r="B61" t="str">
-        <v>Efua Akuffo</v>
+        <v>Akua Quaye</v>
       </c>
       <c r="C61" t="str">
         <v>Parallel Computing</v>
@@ -1440,15 +1440,15 @@
         <v>3</v>
       </c>
       <c r="E61">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>UMaT/PG/0198/24</v>
+        <v>UMaT/PG/0190/24</v>
       </c>
       <c r="B62" t="str">
-        <v>Adwoa Amoah</v>
+        <v>Adjoa Ofori</v>
       </c>
       <c r="C62" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1457,15 +1457,15 @@
         <v>3</v>
       </c>
       <c r="E62">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>UMaT/PG/0198/24</v>
+        <v>UMaT/PG/0190/24</v>
       </c>
       <c r="B63" t="str">
-        <v>Adwoa Amoah</v>
+        <v>Adjoa Ofori</v>
       </c>
       <c r="C63" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1474,15 +1474,15 @@
         <v>3</v>
       </c>
       <c r="E63">
-        <v>65</v>
+        <v>53</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>UMaT/PG/0198/24</v>
+        <v>UMaT/PG/0190/24</v>
       </c>
       <c r="B64" t="str">
-        <v>Adwoa Amoah</v>
+        <v>Adjoa Ofori</v>
       </c>
       <c r="C64" t="str">
         <v>Realtime Systems</v>
@@ -1491,15 +1491,15 @@
         <v>3</v>
       </c>
       <c r="E64">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>UMaT/PG/0198/24</v>
+        <v>UMaT/PG/0190/24</v>
       </c>
       <c r="B65" t="str">
-        <v>Adwoa Amoah</v>
+        <v>Adjoa Ofori</v>
       </c>
       <c r="C65" t="str">
         <v>Parallel Computing</v>
@@ -1508,15 +1508,15 @@
         <v>3</v>
       </c>
       <c r="E65">
-        <v>71</v>
+        <v>61</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>UMaT/PG/0205/24</v>
+        <v>UMaT/PG/0210/24</v>
       </c>
       <c r="B66" t="str">
-        <v>Akua Agyei</v>
+        <v>Kwadwo Quaye</v>
       </c>
       <c r="C66" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1525,15 +1525,15 @@
         <v>3</v>
       </c>
       <c r="E66">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>UMaT/PG/0205/24</v>
+        <v>UMaT/PG/0210/24</v>
       </c>
       <c r="B67" t="str">
-        <v>Akua Agyei</v>
+        <v>Kwadwo Quaye</v>
       </c>
       <c r="C67" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1542,15 +1542,15 @@
         <v>3</v>
       </c>
       <c r="E67">
-        <v>77</v>
+        <v>49</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>UMaT/PG/0205/24</v>
+        <v>UMaT/PG/0210/24</v>
       </c>
       <c r="B68" t="str">
-        <v>Akua Agyei</v>
+        <v>Kwadwo Quaye</v>
       </c>
       <c r="C68" t="str">
         <v>Realtime Systems</v>
@@ -1559,15 +1559,15 @@
         <v>3</v>
       </c>
       <c r="E68">
-        <v>73</v>
+        <v>61</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>UMaT/PG/0205/24</v>
+        <v>UMaT/PG/0210/24</v>
       </c>
       <c r="B69" t="str">
-        <v>Akua Agyei</v>
+        <v>Kwadwo Quaye</v>
       </c>
       <c r="C69" t="str">
         <v>Parallel Computing</v>
@@ -1576,15 +1576,15 @@
         <v>3</v>
       </c>
       <c r="E69">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>UMaT/PG/0216/24</v>
+        <v>UMaT/PG/0217/24</v>
       </c>
       <c r="B70" t="str">
-        <v>Kwadwo Annan</v>
+        <v>Araba Asante</v>
       </c>
       <c r="C70" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1593,15 +1593,15 @@
         <v>3</v>
       </c>
       <c r="E70">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>UMaT/PG/0216/24</v>
+        <v>UMaT/PG/0217/24</v>
       </c>
       <c r="B71" t="str">
-        <v>Kwadwo Annan</v>
+        <v>Araba Asante</v>
       </c>
       <c r="C71" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1610,15 +1610,15 @@
         <v>3</v>
       </c>
       <c r="E71">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>UMaT/PG/0216/24</v>
+        <v>UMaT/PG/0217/24</v>
       </c>
       <c r="B72" t="str">
-        <v>Kwadwo Annan</v>
+        <v>Araba Asante</v>
       </c>
       <c r="C72" t="str">
         <v>Realtime Systems</v>
@@ -1627,15 +1627,15 @@
         <v>3</v>
       </c>
       <c r="E72">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>UMaT/PG/0216/24</v>
+        <v>UMaT/PG/0217/24</v>
       </c>
       <c r="B73" t="str">
-        <v>Kwadwo Annan</v>
+        <v>Araba Asante</v>
       </c>
       <c r="C73" t="str">
         <v>Parallel Computing</v>
@@ -1644,15 +1644,15 @@
         <v>3</v>
       </c>
       <c r="E73">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>UMaT/PG/0239/24</v>
+        <v>UMaT/PG/0222/24</v>
       </c>
       <c r="B74" t="str">
-        <v>Ekua Mensah</v>
+        <v>Kwadwo Ofori</v>
       </c>
       <c r="C74" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1661,15 +1661,15 @@
         <v>3</v>
       </c>
       <c r="E74">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>UMaT/PG/0239/24</v>
+        <v>UMaT/PG/0222/24</v>
       </c>
       <c r="B75" t="str">
-        <v>Ekua Mensah</v>
+        <v>Kwadwo Ofori</v>
       </c>
       <c r="C75" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1678,15 +1678,15 @@
         <v>3</v>
       </c>
       <c r="E75">
-        <v>40</v>
+        <v>67</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>UMaT/PG/0239/24</v>
+        <v>UMaT/PG/0222/24</v>
       </c>
       <c r="B76" t="str">
-        <v>Ekua Mensah</v>
+        <v>Kwadwo Ofori</v>
       </c>
       <c r="C76" t="str">
         <v>Realtime Systems</v>
@@ -1695,15 +1695,15 @@
         <v>3</v>
       </c>
       <c r="E76">
-        <v>57</v>
+        <v>79</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>UMaT/PG/0239/24</v>
+        <v>UMaT/PG/0222/24</v>
       </c>
       <c r="B77" t="str">
-        <v>Ekua Mensah</v>
+        <v>Kwadwo Ofori</v>
       </c>
       <c r="C77" t="str">
         <v>Parallel Computing</v>
@@ -1712,15 +1712,15 @@
         <v>3</v>
       </c>
       <c r="E77">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>UMaT/PG/0242/24</v>
+        <v>UMaT/PG/0236/24</v>
       </c>
       <c r="B78" t="str">
-        <v>Kodwo Frimpong</v>
+        <v>Kobina Frimpong</v>
       </c>
       <c r="C78" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1734,10 +1734,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>UMaT/PG/0242/24</v>
+        <v>UMaT/PG/0236/24</v>
       </c>
       <c r="B79" t="str">
-        <v>Kodwo Frimpong</v>
+        <v>Kobina Frimpong</v>
       </c>
       <c r="C79" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1746,15 +1746,15 @@
         <v>3</v>
       </c>
       <c r="E79">
-        <v>78</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>UMaT/PG/0242/24</v>
+        <v>UMaT/PG/0236/24</v>
       </c>
       <c r="B80" t="str">
-        <v>Kodwo Frimpong</v>
+        <v>Kobina Frimpong</v>
       </c>
       <c r="C80" t="str">
         <v>Realtime Systems</v>
@@ -1763,15 +1763,15 @@
         <v>3</v>
       </c>
       <c r="E80">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>UMaT/PG/0242/24</v>
+        <v>UMaT/PG/0236/24</v>
       </c>
       <c r="B81" t="str">
-        <v>Kodwo Frimpong</v>
+        <v>Kobina Frimpong</v>
       </c>
       <c r="C81" t="str">
         <v>Parallel Computing</v>
@@ -1780,15 +1780,15 @@
         <v>3</v>
       </c>
       <c r="E81">
-        <v>82</v>
+        <v>62</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>UMaT/PG/0248/24</v>
+        <v>UMaT/PG/0244/24</v>
       </c>
       <c r="B82" t="str">
-        <v>Kodwo Sarpong</v>
+        <v>Akosua Afriyie</v>
       </c>
       <c r="C82" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1797,15 +1797,15 @@
         <v>3</v>
       </c>
       <c r="E82">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>UMaT/PG/0248/24</v>
+        <v>UMaT/PG/0244/24</v>
       </c>
       <c r="B83" t="str">
-        <v>Kodwo Sarpong</v>
+        <v>Akosua Afriyie</v>
       </c>
       <c r="C83" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1814,15 +1814,15 @@
         <v>3</v>
       </c>
       <c r="E83">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>UMaT/PG/0248/24</v>
+        <v>UMaT/PG/0244/24</v>
       </c>
       <c r="B84" t="str">
-        <v>Kodwo Sarpong</v>
+        <v>Akosua Afriyie</v>
       </c>
       <c r="C84" t="str">
         <v>Realtime Systems</v>
@@ -1831,15 +1831,15 @@
         <v>3</v>
       </c>
       <c r="E84">
-        <v>77</v>
+        <v>86</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>UMaT/PG/0248/24</v>
+        <v>UMaT/PG/0244/24</v>
       </c>
       <c r="B85" t="str">
-        <v>Kodwo Sarpong</v>
+        <v>Akosua Afriyie</v>
       </c>
       <c r="C85" t="str">
         <v>Parallel Computing</v>
@@ -1848,15 +1848,15 @@
         <v>3</v>
       </c>
       <c r="E85">
-        <v>77</v>
+        <v>63</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>UMaT/PG/0253/24</v>
+        <v>UMaT/PG/0261/24</v>
       </c>
       <c r="B86" t="str">
-        <v>Kwame Danquah</v>
+        <v>Kwadwo Acheampong</v>
       </c>
       <c r="C86" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1865,15 +1865,15 @@
         <v>3</v>
       </c>
       <c r="E86">
-        <v>73</v>
+        <v>100</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>UMaT/PG/0253/24</v>
+        <v>UMaT/PG/0261/24</v>
       </c>
       <c r="B87" t="str">
-        <v>Kwame Danquah</v>
+        <v>Kwadwo Acheampong</v>
       </c>
       <c r="C87" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1882,15 +1882,15 @@
         <v>3</v>
       </c>
       <c r="E87">
-        <v>77</v>
+        <v>68</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>UMaT/PG/0253/24</v>
+        <v>UMaT/PG/0261/24</v>
       </c>
       <c r="B88" t="str">
-        <v>Kwame Danquah</v>
+        <v>Kwadwo Acheampong</v>
       </c>
       <c r="C88" t="str">
         <v>Realtime Systems</v>
@@ -1899,15 +1899,15 @@
         <v>3</v>
       </c>
       <c r="E88">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>UMaT/PG/0253/24</v>
+        <v>UMaT/PG/0261/24</v>
       </c>
       <c r="B89" t="str">
-        <v>Kwame Danquah</v>
+        <v>Kwadwo Acheampong</v>
       </c>
       <c r="C89" t="str">
         <v>Parallel Computing</v>
@@ -1916,15 +1916,15 @@
         <v>3</v>
       </c>
       <c r="E89">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>UMaT/PG/0259/24</v>
+        <v>UMaT/PG/0275/24</v>
       </c>
       <c r="B90" t="str">
-        <v>Kwame Nkrumah</v>
+        <v>Araba Amoah</v>
       </c>
       <c r="C90" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -1933,15 +1933,15 @@
         <v>3</v>
       </c>
       <c r="E90">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>UMaT/PG/0259/24</v>
+        <v>UMaT/PG/0275/24</v>
       </c>
       <c r="B91" t="str">
-        <v>Kwame Nkrumah</v>
+        <v>Araba Amoah</v>
       </c>
       <c r="C91" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -1950,15 +1950,15 @@
         <v>3</v>
       </c>
       <c r="E91">
-        <v>78</v>
+        <v>50</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>UMaT/PG/0259/24</v>
+        <v>UMaT/PG/0275/24</v>
       </c>
       <c r="B92" t="str">
-        <v>Kwame Nkrumah</v>
+        <v>Araba Amoah</v>
       </c>
       <c r="C92" t="str">
         <v>Realtime Systems</v>
@@ -1967,15 +1967,15 @@
         <v>3</v>
       </c>
       <c r="E92">
-        <v>61</v>
+        <v>50</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>UMaT/PG/0259/24</v>
+        <v>UMaT/PG/0275/24</v>
       </c>
       <c r="B93" t="str">
-        <v>Kwame Nkrumah</v>
+        <v>Araba Amoah</v>
       </c>
       <c r="C93" t="str">
         <v>Parallel Computing</v>
@@ -1984,15 +1984,15 @@
         <v>3</v>
       </c>
       <c r="E93">
-        <v>54</v>
+        <v>78</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>UMaT/PG/0270/24</v>
+        <v>UMaT/PG/0280/24</v>
       </c>
       <c r="B94" t="str">
-        <v>Abena Acheampong</v>
+        <v>Akosua Darko</v>
       </c>
       <c r="C94" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -2001,15 +2001,15 @@
         <v>3</v>
       </c>
       <c r="E94">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>UMaT/PG/0270/24</v>
+        <v>UMaT/PG/0280/24</v>
       </c>
       <c r="B95" t="str">
-        <v>Abena Acheampong</v>
+        <v>Akosua Darko</v>
       </c>
       <c r="C95" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -2018,15 +2018,15 @@
         <v>3</v>
       </c>
       <c r="E95">
-        <v>52</v>
+        <v>65</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>UMaT/PG/0270/24</v>
+        <v>UMaT/PG/0280/24</v>
       </c>
       <c r="B96" t="str">
-        <v>Abena Acheampong</v>
+        <v>Akosua Darko</v>
       </c>
       <c r="C96" t="str">
         <v>Realtime Systems</v>
@@ -2035,15 +2035,15 @@
         <v>3</v>
       </c>
       <c r="E96">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>UMaT/PG/0270/24</v>
+        <v>UMaT/PG/0280/24</v>
       </c>
       <c r="B97" t="str">
-        <v>Abena Acheampong</v>
+        <v>Akosua Darko</v>
       </c>
       <c r="C97" t="str">
         <v>Parallel Computing</v>
@@ -2052,15 +2052,15 @@
         <v>3</v>
       </c>
       <c r="E97">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>UMaT/PG/0275/24</v>
+        <v>UMaT/PG/0283/24</v>
       </c>
       <c r="B98" t="str">
-        <v>Kakra Amankwah</v>
+        <v>Araba Agyemang</v>
       </c>
       <c r="C98" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -2069,15 +2069,15 @@
         <v>3</v>
       </c>
       <c r="E98">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>UMaT/PG/0275/24</v>
+        <v>UMaT/PG/0283/24</v>
       </c>
       <c r="B99" t="str">
-        <v>Kakra Amankwah</v>
+        <v>Araba Agyemang</v>
       </c>
       <c r="C99" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -2086,15 +2086,15 @@
         <v>3</v>
       </c>
       <c r="E99">
-        <v>73</v>
+        <v>58</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>UMaT/PG/0275/24</v>
+        <v>UMaT/PG/0283/24</v>
       </c>
       <c r="B100" t="str">
-        <v>Kakra Amankwah</v>
+        <v>Araba Agyemang</v>
       </c>
       <c r="C100" t="str">
         <v>Realtime Systems</v>
@@ -2103,15 +2103,15 @@
         <v>3</v>
       </c>
       <c r="E100">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>UMaT/PG/0275/24</v>
+        <v>UMaT/PG/0283/24</v>
       </c>
       <c r="B101" t="str">
-        <v>Kakra Amankwah</v>
+        <v>Araba Agyemang</v>
       </c>
       <c r="C101" t="str">
         <v>Parallel Computing</v>
@@ -2120,15 +2120,15 @@
         <v>3</v>
       </c>
       <c r="E101">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>UMaT/PG/0284/24</v>
+        <v>UMaT/PG/0292/24</v>
       </c>
       <c r="B102" t="str">
-        <v>Yaa Akuffo</v>
+        <v>Adwoa Adjei</v>
       </c>
       <c r="C102" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -2137,15 +2137,15 @@
         <v>3</v>
       </c>
       <c r="E102">
-        <v>77</v>
+        <v>53</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>UMaT/PG/0284/24</v>
+        <v>UMaT/PG/0292/24</v>
       </c>
       <c r="B103" t="str">
-        <v>Yaa Akuffo</v>
+        <v>Adwoa Adjei</v>
       </c>
       <c r="C103" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -2154,15 +2154,15 @@
         <v>3</v>
       </c>
       <c r="E103">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>UMaT/PG/0284/24</v>
+        <v>UMaT/PG/0292/24</v>
       </c>
       <c r="B104" t="str">
-        <v>Yaa Akuffo</v>
+        <v>Adwoa Adjei</v>
       </c>
       <c r="C104" t="str">
         <v>Realtime Systems</v>
@@ -2171,15 +2171,15 @@
         <v>3</v>
       </c>
       <c r="E104">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>UMaT/PG/0284/24</v>
+        <v>UMaT/PG/0292/24</v>
       </c>
       <c r="B105" t="str">
-        <v>Yaa Akuffo</v>
+        <v>Adwoa Adjei</v>
       </c>
       <c r="C105" t="str">
         <v>Parallel Computing</v>
@@ -2188,15 +2188,15 @@
         <v>3</v>
       </c>
       <c r="E105">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>UMaT/PG/0298/24</v>
+        <v>UMaT/PG/0296/24</v>
       </c>
       <c r="B106" t="str">
-        <v>Kojo Osei</v>
+        <v>Kofi Opoku</v>
       </c>
       <c r="C106" t="str">
         <v>Very Large Scale Integration (VLSI)</v>
@@ -2205,15 +2205,15 @@
         <v>3</v>
       </c>
       <c r="E106">
-        <v>93</v>
+        <v>48</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>UMaT/PG/0298/24</v>
+        <v>UMaT/PG/0296/24</v>
       </c>
       <c r="B107" t="str">
-        <v>Kojo Osei</v>
+        <v>Kofi Opoku</v>
       </c>
       <c r="C107" t="str">
         <v>Optimisation Methods and Applications</v>
@@ -2222,15 +2222,15 @@
         <v>3</v>
       </c>
       <c r="E107">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>UMaT/PG/0298/24</v>
+        <v>UMaT/PG/0296/24</v>
       </c>
       <c r="B108" t="str">
-        <v>Kojo Osei</v>
+        <v>Kofi Opoku</v>
       </c>
       <c r="C108" t="str">
         <v>Realtime Systems</v>
@@ -2239,15 +2239,15 @@
         <v>3</v>
       </c>
       <c r="E108">
-        <v>98</v>
+        <v>48</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>UMaT/PG/0298/24</v>
+        <v>UMaT/PG/0296/24</v>
       </c>
       <c r="B109" t="str">
-        <v>Kojo Osei</v>
+        <v>Kofi Opoku</v>
       </c>
       <c r="C109" t="str">
         <v>Parallel Computing</v>
@@ -2256,7 +2256,7 @@
         <v>3</v>
       </c>
       <c r="E109">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>